<commit_message>
Remove Moyle interconnector policy; scenarios include import and export
</commit_message>
<xml_diff>
--- a/data/policy_uplift.xlsx
+++ b/data/policy_uplift.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://people.ey.com/personal/minoo_ashoori_ie_ey_com/Documents/Desktop/SIB/whole_picture_2/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://people.ey.com/personal/minoo_ashoori_ie_ey_com/Documents/Desktop/SIB/Energy_80_by_2030/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="340" documentId="8_{9BAEE778-95C0-4FC3-8C1F-75F0B4E9362D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84B6BCDE-9D86-43E1-A514-64A1B484FA4F}"/>
+  <xr:revisionPtr revIDLastSave="358" documentId="8_{9BAEE778-95C0-4FC3-8C1F-75F0B4E9362D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87DFE9B6-9981-4C85-9B1F-C0E49E1CCAED}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="5" xr2:uid="{83ACEBD2-7A49-4900-9217-34DAFC24AD63}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="4" xr2:uid="{83ACEBD2-7A49-4900-9217-34DAFC24AD63}"/>
   </bookViews>
   <sheets>
     <sheet name="all" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="19">
   <si>
     <t>Policy</t>
   </si>
@@ -1906,7 +1906,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{400E2126-E6E4-431E-9468-62D593B8CE37}">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.26953125" bestFit="1" customWidth="1"/>
@@ -2009,11 +2009,11 @@
         <v>35808840.688000001</v>
       </c>
       <c r="E4">
-        <f t="shared" ref="E3:E11" si="0">C4/D4</f>
+        <f t="shared" ref="E4:E9" si="0">C4/D4</f>
         <v>0.44369799913608415</v>
       </c>
       <c r="F4">
-        <f t="shared" ref="F4:F11" si="1">C4-$C$2</f>
+        <f t="shared" ref="F4:F9" si="1">C4-$C$2</f>
         <v>3196734.8206054997</v>
       </c>
       <c r="G4">
@@ -2024,7 +2024,7 @@
         <v>9620709.7319374997</v>
       </c>
       <c r="I4">
-        <f t="shared" ref="I4:I11" si="2">(H4-$H$2)/$H$2</f>
+        <f t="shared" ref="I4:I10" si="2">(H4-$H$2)/$H$2</f>
         <v>-0.24940500483547548</v>
       </c>
     </row>
@@ -2063,195 +2063,163 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="C6">
-        <v>12691576.1440429</v>
+        <v>15952249.779492101</v>
       </c>
       <c r="D6">
         <v>35808840.688000001</v>
       </c>
       <c r="E6">
-        <f t="shared" si="0"/>
-        <v>0.35442577587539742</v>
+        <f>C6/D6</f>
+        <v>0.44548355861288474</v>
       </c>
       <c r="F6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3260673.6354492009</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <f t="shared" ref="G6:G8" si="3">E6-$E$2</f>
+        <v>9.105778273253845E-2</v>
       </c>
       <c r="H6">
-        <v>12817444.552542901</v>
+        <v>9556770.9170937501</v>
       </c>
       <c r="I6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-0.2543934262467516</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B7">
-        <v>2027</v>
+        <v>2029</v>
       </c>
       <c r="C7">
-        <v>15952249.779492101</v>
+        <v>14401388.273925699</v>
       </c>
       <c r="D7">
         <v>35808840.688000001</v>
       </c>
       <c r="E7">
-        <f>C7/D7</f>
-        <v>0.44548355861288474</v>
+        <f t="shared" si="0"/>
+        <v>0.40217409994933984</v>
       </c>
       <c r="F7">
         <f t="shared" si="1"/>
-        <v>3260673.6354492009</v>
+        <v>1709812.1298827995</v>
       </c>
       <c r="G7">
-        <f t="shared" ref="G4:G10" si="3">E7-$E$2</f>
-        <v>9.105778273253845E-2</v>
+        <f t="shared" si="3"/>
+        <v>4.7748324068993542E-2</v>
       </c>
       <c r="H7">
-        <v>9556770.9170937501</v>
+        <v>11107632.422660099</v>
       </c>
       <c r="I7">
         <f t="shared" si="2"/>
-        <v>-0.2543934262467516</v>
+        <v>-0.13339727141972191</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B8">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="C8">
-        <v>14401388.273925699</v>
+        <v>13084420.169384699</v>
       </c>
       <c r="D8">
         <v>35808840.688000001</v>
       </c>
       <c r="E8">
         <f t="shared" si="0"/>
-        <v>0.40217409994933984</v>
+        <v>0.36539636352342048</v>
       </c>
       <c r="F8">
         <f t="shared" si="1"/>
-        <v>1709812.1298827995</v>
+        <v>392844.02534179948</v>
       </c>
       <c r="G8">
         <f t="shared" si="3"/>
-        <v>4.7748324068993542E-2</v>
+        <v>1.0970587643074181E-2</v>
       </c>
       <c r="H8">
-        <v>11107632.422660099</v>
+        <v>12424600.527201099</v>
       </c>
       <c r="I8">
         <f t="shared" si="2"/>
-        <v>-0.13339727141972191</v>
+        <v>-3.0649169086037788E-2</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B9">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="C9">
-        <v>13084420.169384699</v>
+        <v>12691576.1440429</v>
       </c>
       <c r="D9">
         <v>35808840.688000001</v>
       </c>
       <c r="E9">
         <f t="shared" si="0"/>
-        <v>0.36539636352342048</v>
+        <v>0.35442577587539742</v>
       </c>
       <c r="F9">
         <f t="shared" si="1"/>
-        <v>392844.02534179948</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <f t="shared" si="3"/>
-        <v>1.0970587643074181E-2</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>12424600.527201099</v>
+        <v>12817444.552542901</v>
       </c>
       <c r="I9">
         <f t="shared" si="2"/>
-        <v>-3.0649169086037788E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10">
-        <v>2031</v>
+        <v>14</v>
       </c>
       <c r="C10">
-        <v>12691576.1440429</v>
+        <v>18352682.007874999</v>
       </c>
       <c r="D10">
         <v>35808840.688000001</v>
       </c>
       <c r="E10">
-        <f t="shared" si="0"/>
-        <v>0.35442577587539742</v>
-      </c>
-      <c r="F10">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>C10/D10</f>
+        <v>0.51251818420430506</v>
+      </c>
+      <c r="F10" s="1">
+        <f>C10-$C$2</f>
+        <v>5661105.8638320994</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <f>E10-$E$2</f>
+        <v>0.15809240832395877</v>
       </c>
       <c r="H10">
-        <v>12817444.552542901</v>
+        <v>7156338.6887109298</v>
       </c>
       <c r="I10">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11">
-        <v>24754397.155675702</v>
-      </c>
-      <c r="D11">
-        <v>35808840.688000001</v>
-      </c>
-      <c r="E11">
-        <f>C11/D11</f>
-        <v>0.69129289527575288</v>
-      </c>
-      <c r="F11">
-        <f t="shared" si="1"/>
-        <v>12062821.011632802</v>
-      </c>
-      <c r="G11">
-        <f>E11-$E$2</f>
-        <v>0.33686711939540659</v>
-      </c>
-      <c r="H11">
-        <v>754623.54091015598</v>
-      </c>
-      <c r="I11">
-        <f t="shared" si="2"/>
-        <v>-0.94112527362090725</v>
+        <v>-0.44167196047739821</v>
       </c>
     </row>
   </sheetData>
@@ -2262,7 +2230,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E4FF95A-5103-44A8-A361-01717069412F}">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.26953125" bestFit="1" customWidth="1"/>
@@ -2362,11 +2330,11 @@
         <v>36080210.625</v>
       </c>
       <c r="E4">
-        <f t="shared" ref="E4:E11" si="0">C4/D4</f>
+        <f t="shared" ref="E4:E9" si="0">C4/D4</f>
         <v>0.40700341275041824</v>
       </c>
       <c r="F4">
-        <f t="shared" ref="F4:F11" si="1">C4-$C$2</f>
+        <f t="shared" ref="F4:F9" si="1">C4-$C$2</f>
         <v>3222150.4269532003</v>
       </c>
       <c r="G4">
@@ -2377,7 +2345,7 @@
         <v>11786016.023050699</v>
       </c>
       <c r="I4">
-        <f t="shared" ref="I4:I11" si="2">(H4-$H$2)/$H$2</f>
+        <f t="shared" ref="I4:I9" si="2">(H4-$H$2)/$H$2</f>
         <v>-0.21469314307560622</v>
       </c>
     </row>
@@ -2416,195 +2384,163 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="C6">
-        <v>11462618.430175699</v>
+        <v>14803099.3731445</v>
       </c>
       <c r="D6">
         <v>36080210.625</v>
       </c>
       <c r="E6">
-        <f t="shared" si="0"/>
-        <v>0.3176982127214425</v>
+        <f>C6/D6</f>
+        <v>0.41028306422600047</v>
       </c>
       <c r="F6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3340480.9429688007</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <f>E6-$E$2</f>
+        <v>9.2584851504557975E-2</v>
       </c>
       <c r="H6">
-        <v>15008166.4500039</v>
+        <v>11667685.507035101</v>
       </c>
       <c r="I6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-0.22257755163475887</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B7">
-        <v>2027</v>
+        <v>2029</v>
       </c>
       <c r="C7">
-        <v>14803099.3731445</v>
+        <v>13190618.430175699</v>
       </c>
       <c r="D7">
         <v>36080210.625</v>
       </c>
       <c r="E7">
-        <f>C7/D7</f>
-        <v>0.41028306422600047</v>
+        <f t="shared" si="0"/>
+        <v>0.3655915029785306</v>
       </c>
       <c r="F7">
         <f t="shared" si="1"/>
-        <v>3340480.9429688007</v>
+        <v>1728000</v>
       </c>
       <c r="G7">
-        <f>E7-$E$2</f>
-        <v>9.2584851504557975E-2</v>
+        <f t="shared" ref="G7" si="3">E7-$E$2</f>
+        <v>4.7893290257088106E-2</v>
       </c>
       <c r="H7">
-        <v>11667685.507035101</v>
+        <v>13280166.4500039</v>
       </c>
       <c r="I7">
         <f t="shared" si="2"/>
-        <v>-0.22257755163475887</v>
+        <v>-0.1151373157911339</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B8">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="C8">
-        <v>13190618.430175699</v>
+        <v>11923980.902587799</v>
       </c>
       <c r="D8">
         <v>36080210.625</v>
       </c>
       <c r="E8">
-        <f t="shared" si="0"/>
-        <v>0.3655915029785306</v>
+        <f>C8/D8</f>
+        <v>0.33048534628912796</v>
       </c>
       <c r="F8">
         <f t="shared" si="1"/>
-        <v>1728000</v>
+        <v>461362.47241210006</v>
       </c>
       <c r="G8">
-        <f t="shared" ref="G7:G11" si="3">E8-$E$2</f>
-        <v>4.7893290257088106E-2</v>
+        <f>E8-$E$2</f>
+        <v>1.278713356768546E-2</v>
       </c>
       <c r="H8">
-        <v>13280166.4500039</v>
+        <v>14546803.9775918</v>
       </c>
       <c r="I8">
         <f t="shared" si="2"/>
-        <v>-0.1151373157911339</v>
+        <v>-3.0740761967760571E-2</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B9">
-        <v>2030</v>
-      </c>
-      <c r="C9">
-        <v>11923980.902587799</v>
+        <v>2031</v>
+      </c>
+      <c r="C9" s="1">
+        <v>11462618.430175699</v>
       </c>
       <c r="D9">
         <v>36080210.625</v>
       </c>
       <c r="E9">
-        <f>C9/D9</f>
-        <v>0.33048534628912796</v>
+        <f t="shared" si="0"/>
+        <v>0.3176982127214425</v>
       </c>
       <c r="F9">
         <f t="shared" si="1"/>
-        <v>461362.47241210006</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <f>E9-$E$2</f>
-        <v>1.278713356768546E-2</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>14546803.9775918</v>
+        <v>15008166.4500039</v>
       </c>
       <c r="I9">
         <f t="shared" si="2"/>
-        <v>-3.0740761967760571E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10">
-        <v>2031</v>
-      </c>
-      <c r="C10" s="1">
-        <v>11462618.430175699</v>
+        <v>14</v>
+      </c>
+      <c r="C10">
+        <v>17706806.253125001</v>
       </c>
       <c r="D10">
         <v>36080210.625</v>
       </c>
       <c r="E10">
-        <f t="shared" si="0"/>
-        <v>0.3176982127214425</v>
-      </c>
-      <c r="F10">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>C10/D10</f>
+        <v>0.49076227511975618</v>
+      </c>
+      <c r="F10" s="1">
+        <f>C10-$C$2</f>
+        <v>6244187.8229493015</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <f>E10-$E$2</f>
+        <v>0.17306406239831368</v>
       </c>
       <c r="H10">
-        <v>15008166.4500039</v>
+        <v>5875631.6755742095</v>
       </c>
       <c r="I10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11">
-        <v>24514179.167515598</v>
-      </c>
-      <c r="D11">
-        <v>36080210.625</v>
-      </c>
-      <c r="E11">
-        <f>C11/D11</f>
-        <v>0.67943558928477288</v>
-      </c>
-      <c r="F11">
-        <f t="shared" si="1"/>
-        <v>13051560.737339899</v>
-      </c>
-      <c r="G11">
-        <f>E11-$E$2</f>
-        <v>0.36173737656333038</v>
-      </c>
-      <c r="H11">
-        <v>1956605.7126640601</v>
-      </c>
-      <c r="I11">
-        <f t="shared" si="2"/>
-        <v>-0.86963059617029026</v>
+        <f>(H10-$H$2)/$H$2</f>
+        <v>-0.60850436359781424</v>
       </c>
     </row>
   </sheetData>

</xml_diff>